<commit_message>
add PCS model in simulink library
</commit_message>
<xml_diff>
--- a/Examples/AcPowerSystem/SingleApparatusInfiniteBus/GfmInverterInfiniteBus.xlsx
+++ b/Examples/AcPowerSystem/SingleApparatusInfiniteBus/GfmInverterInfiniteBus.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\liao\Desktop\毕业设计\Simplus-Grid-Tool\Examples\AcPowerSystem\SingleApparatusInfiniteBus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F96DE7B-8173-497A-AC0F-4D2D2B199F85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E050031E-3A96-4148-A1AF-A44E5E6B6ABE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bus" sheetId="1" r:id="rId1"/>
@@ -837,7 +837,7 @@
         <v>2</v>
       </c>
       <c r="B5">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C5" s="2">
         <v>0.05</v>
@@ -1155,7 +1155,7 @@
         <v>35</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
Add battery and photovoltaic system, modify interlink ACDC control mode
</commit_message>
<xml_diff>
--- a/Examples/AcPowerSystem/SingleApparatusInfiniteBus/GfmInverterInfiniteBus.xlsx
+++ b/Examples/AcPowerSystem/SingleApparatusInfiniteBus/GfmInverterInfiniteBus.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Power-System-Analysis-Toolbox\Examples\AcPowerSystem\SingleApparatusInfiniteBus\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Research\Simplus-Grid-Tool-Merge\Simplus-Grid-Tool\Examples\AcPowerSystem\SingleApparatusInfiniteBus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ECE420B-1BDE-4F00-AF39-9DFAC6740526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF981DA3-30E5-4FAC-AD33-6C750CA048CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-90" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bus" sheetId="1" r:id="rId1"/>
@@ -20,18 +20,10 @@
     <sheet name="Basic" sheetId="4" r:id="rId5"/>
     <sheet name="Advance" sheetId="6" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -315,7 +307,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>

</xml_diff>

<commit_message>
Fix variable naming issues
</commit_message>
<xml_diff>
--- a/Examples/AcPowerSystem/SingleApparatusInfiniteBus/GfmInverterInfiniteBus.xlsx
+++ b/Examples/AcPowerSystem/SingleApparatusInfiniteBus/GfmInverterInfiniteBus.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Research\Simplus-Grid-Tool-Merge\Simplus-Grid-Tool\Examples\AcPowerSystem\SingleApparatusInfiniteBus\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Power-System-Analysis-Toolbox\Examples\AcPowerSystem\SingleApparatusInfiniteBus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF981DA3-30E5-4FAC-AD33-6C750CA048CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ECE420B-1BDE-4F00-AF39-9DFAC6740526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-90" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bus" sheetId="1" r:id="rId1"/>
@@ -20,10 +20,18 @@
     <sheet name="Basic" sheetId="4" r:id="rId5"/>
     <sheet name="Advance" sheetId="6" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -307,7 +315,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>

</xml_diff>